<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 3, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -445,10 +445,797 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>큐텐상품번호</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>상점ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>상품명(원본)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>한글검증명칭</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>가격(엔)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>리뷰수</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>옵션있음</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>카테고리코드</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>상품URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1203566602</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>vanguardvista</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[正規品1+1] ヒートアクティブ極損傷傷つけるトリートメント 220ml+220ml</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2891</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203566602</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1031781330</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>gugumile</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[5枚] ナンバーズイン 4番 SOS急速冷却シートマスク, 27g*5 マスクシート</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1572</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1031781330</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>997222280</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>gugumile</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ビフィダ バイオーム コンセントレート クリーム50ml/韓国化粧品/スキンケア/クリーム</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>3465</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=997222280</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1141816688</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>JDKM</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>トーンアップ ホワイト マッド マスク 3個入り x 2個</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>バイアウア</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>5214</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141816688</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1141816327</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>JDKM</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>わさびスージングマスク 30g</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Miss Dragon</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>5709</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141816327</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1191488311</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>hmipo</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>アクアティカ サンスプレー 100mL</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191488311</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1206876054</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>NARShA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>[ブラシ元祖] グロウターンエクソソームブラシアンプル130ml企画(+30ml)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>5950</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206876054</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1049588733</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>スーパーヴォルカニックポアクレイマスク2X, 100mL</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1049588733</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1204156842</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>[1+1] トン＆スポット コレクターアンプル 30ml +30ml</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Redence</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>4620</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204156842</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1186174034</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>[1+1]アルガンオイルダメージトリートメント300ml+300ml</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>エラスティン</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>2280</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1186174034</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1156719535</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>modeling</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ソウルシークレットブロッサム香水30ml</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ザフェイスショップ</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>2950</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156719535</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1138185679</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JfromKorea</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>エアリー サンスティック スムージング バー 23g</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>2591</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138185679</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1187136865</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>JfromKorea</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>リアルミルク クレンジングフォーム 肌保湿 弾力 肌のキメ 水分改善150ml1本</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>ブランカウ</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>2863</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187136865</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1177838255</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>JfromKorea</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ハニーアンドマカダミア ネイチャーシャンプー ブラックベリーベイ 500ml</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>2160</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177838255</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1203234617</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>PrincessRamen</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>フォトデルム X-ディフェンス ウルトラ フルイド SPF50+ 40ml</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>ビオデルマ</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>4571</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203234617</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1079657711</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>PrincessRamen</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>トリデン Torriden dive in 低分子 ヒアルロン酸 トナー 300ml/ダイブイントナー 300mL</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1079657711</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1210384893</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PrincessRamen</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ブルー ペプチド バクチオール プランプ バウンス クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>4428</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210384893</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1207603847</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>PrincessRamen</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>メイクアップ フィクサー 80ml</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ヘラ</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>4570</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207603847</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A1"/>
+  <autoFilter ref="A1:J19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 6, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1234,8 +1234,828 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1194335884</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>OneulPick</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>ハイミッシュ マリンケア アイクリーム 30ml (e)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ヘイミッシュ</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>2196</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194335884</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1210847470</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>OneulPick</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>id PLACOSMETICS リアルアフターケアミスト 120ml</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>id PLACOSMETICS</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>3481</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210847470</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1194335721</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>OneulPick</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>タイムレボリューションプライムステム100クリーム50ml</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ミシャ</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>4033</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194335721</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1209978694</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>OneulPick</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ワンレイヤートーンアップボディミスト100ml</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>KAHI</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2495</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209978694</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1138225289</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>dreamus</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>シグネチャーパルファム, 50ml, 1個</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>5517</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1138225289</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1075323842</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>kosmetic</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>THE ORDINARY Alpha Arbutin 2% + HA [KOR] - 30ml</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ザ ヨン</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>3210</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1075323842</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1075016731</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>kosmetic</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>韓国コスメ 肌の保湿The Niacinamide 15 Serum 20ml</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>COSRX</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>2612</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1075016731</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1072484408</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HAMAHAMA</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ダブルユードレスルームドレスパフュームNo.49ピーチブロッサム160ml</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>W.DRESSROOM</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>1700</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1072484408</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1115880952</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HAMAHAMA</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ノースカナイントラブルセラム 30ml</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>パティオン</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>4260</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1115880952</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1072009140</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>バイオ スキン クレンジング パッド 6g 30枚入 x 2</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>EKE</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1072009140</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1083261277</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>KOR--STORE</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>CELL LINE PRO リペアクリーム [100口] 半永久化粧材料 アフターケア 1g100個入り</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Clear_pro</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083261277</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1209979406</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>【正規品】ハンーユル 幼いヨモギ 皮脂吸着 ヨモギ餅パックフォーム 120ml, 1個</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ハンユル</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209979406</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1204386062</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>【正規品】朝鮮の美女 人参アイクリーム 30ml（ビタミンA レチナール リポソーム）</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204386062</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1203715344</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>【正規品】 フォア パーフェクティング コラーゲン ペプチド クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>4190</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203715344</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1202714464</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>【正規品】 マデカーメラキャプチャーアンプルパッド60枚x2個</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202714464</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1204254720</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>k-pick72811</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>[ウォーターミストプランピング][正規品] マダガスカル センテラ ヒアル-テカ プランピング アンプル 50ml／スキンブースティング／ヒアルプラム</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>5743</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204254720</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1199087370</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>k-pick72811</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>[和解1位/脱毛シャンプー] パープルブースター [正規品]玉ねぎシャンプー/紫の抗酸化ブースター</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>prooted</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199087370</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1167124675</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ラエル オーガニックコットンカバー 履くオーバーナイト M 2個入 x3個</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ラエル</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>3059</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167124675</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1202040262</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>ジョソンアビューティ ワンダーバス レモンシロップ パッククレンザー 200ml (+50ml)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>WONDER BATH</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>4332</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202040262</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>1202040223</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>TwoK</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>エストラ エイシカ365 スーディング リペア マスク pH4.5 5枚</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>4378</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202040223</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J19"/>
+  <autoFilter ref="A1:J39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 9, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3202,8 +3202,582 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1210946100</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Yeonbunong</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>オリーブヤング プレステージ ローション トゥエックス ジンセン デスカルゴ 140ml</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>イッツスキン</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>4460</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210946100</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1210829091</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Yeonbunong</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>オリーブヤング ドクターセイバス セラムマスク PDRN 10枚</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>イッツスキン</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>2310</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210829091</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1208091250</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Yeonbunong</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>シグニチャー バイオ ディープ コラーゲン ファーミング マスク パック 12枚入り リフトアップ フェイスパック 韓国コスメ　コラーゲン　ハリ</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>VINNE</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>14500</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208091250</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1199482761</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Yeonbunong</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>[栄養] オリーブヤング 大豆エッセンス 50ml</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ミクスン</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>4570</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199482761</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1208332251</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>hanamiselect</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>【正規品】ライスアクアフレッシュサンクリーム 50ml SPF50+ PA++++ 日焼け止め</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>2190</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208332251</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1208994497</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>hanamiselect</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>【正規品】白樺ミネラルサンクリーム SPF50+ PA++++ 50ml</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>2290</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208994497</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1132391030</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>hanimall</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>アトバリア 365 クリーム 80ml</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>4510</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1132391030</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1146402210</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>hanimall</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>シラカバ 水分 サンクッション 15g</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>3080</v>
+      </c>
+      <c r="G75" t="n">
+        <v>2</v>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146402210</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1133988984</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>hanimall</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>センテッド ハンドクリーム 40ml/韓国化粧品/パフュームハンドクリーム</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>hince</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1133988984</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1211674770</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>KORESHOP</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>ディープダメージリペアシャンプー 500ml + 詰め替え 400ml 大容量セット スイートブリーズの香り</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>4247</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211674770</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1203834476</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>KORESHOP</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>白樺水分サンクッション 15g</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>2109</v>
+      </c>
+      <c r="G78" t="n">
+        <v>3</v>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203834476</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1193418611</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>KVIVE</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>ヒーラー ポア タイトニング トナーパッド 本品60枚+詰め替え用 60枚入り/PDRN トナーパッド 美容液 /韓国 人気 トナーパッド/弾力/保湿/水分アンプル/c-PDRN/エイジングケアトナー</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>リジュラン</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>6870</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193418611</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1202579985</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>KVIVE</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>[1+1] 選べるサンセラム 2個セット (水分鎮静 / 弾力トーンアップ) SPF50+ PA++++/マデカソサイド 鎮静 or PDRN トーンアップ サンセラム / 美容液 日焼けめ</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>メディヒール</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>4890</v>
+      </c>
+      <c r="G80" t="n">
+        <v>1</v>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202579985</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1207120098</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>LUNORASELECT</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>マスターズ エアリッチ サンスティック 22g 2個 セット ポケモン エディション 日焼け止め UVカット 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>4836</v>
+      </c>
+      <c r="G81" t="n">
+        <v>1</v>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207120098</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J67"/>
+  <autoFilter ref="A1:J81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 12, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$96</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3776,8 +3776,623 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1206006286</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ALLisWELL</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ローズオブセッション ティント 24種（グロウ/マット）</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>1831</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206006286</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1197650165</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ALLisWELL</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>EFGセサル軟膏 5g / EGFクリーム (保湿ケア / 敏感肌サポート)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>大熊製薬</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>2548</v>
+      </c>
+      <c r="G83" t="n">
+        <v>3</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197650165</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1194294476</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>myoneshop</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>[マグネティックネイル] マジックプレス グロウベリー（アーモンド）ネイルチップセット 1個</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ダッシングディバ</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>4829</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194294476</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1171937523</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>myoneshop</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>[キンモクセイの香りエディション] ハニーアンドマカダミア ネイチャーパフュームシャンプー400ml×1個+トリートメント400ml×1個+GIFTシャンプーブラシ</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G85" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171937523</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1134929906</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>myoneshop</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>[韓国マスクパックセット]ダイブイン低分子ヒアルロン酸マスク6枚+メディヒールマデカソサイドエッセンシャルマスク11枚+GIFTナンバーズイン2番ビューティーコラーゲンボリュープマスク1枚</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>トリデン</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>6299</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134929906</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1207547885</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>kim701016</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>メラノサクリーム 30g</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>東亜製薬</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207547885</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1204931350</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>kim701016</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>スーパー ドロップス - ビタC トーニング セラム 大容量バナナキック エディション</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>ビリーフ</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>4050</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="b">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204931350</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1204628544</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>kim701016</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ハウス・オブ・ビ・グルタチオン・フェイスフィルム（3+1）</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>HOUSE OF B</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>5400</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204628544</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1203899937</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>kim701016</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>レッドサクセニックアシッドパッド/ ニキビ跡・角質ケア・毛穴汚れ / 低刺激・拭き取り化粧水</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203899937</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1203826917</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>kim701016</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>ヒアルロン酸水分カプセルクリーム 55g/インナードライ・保湿・ツヤ肌 / 低刺激・水分補給</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>3960</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="b">
+        <v>0</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203826917</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1191781202</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>MEDIHEAL トナーパッド2.0 リフィル 70枚×2個セット 4タイプ選択可</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>1918</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="b">
+        <v>0</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191781202</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1204359324</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>A-RAUM</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>【1+1 / SNS話題】ツヤ肌バブルエッセンストナー 95ml</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>curest</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>2131</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="b">
+        <v>0</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204359324</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1120129564</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ikoniko</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>ヘアロールブラシ(Big,58mm)ヘアスタイリング</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>HAUM</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>4475</v>
+      </c>
+      <c r="G94" t="n">
+        <v>2</v>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1120129564</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1151670543</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>KORKORMALL</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>[国内百貨店]ディープディックフレッドポッドボディバーム200ml</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>ディプティック</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>16500</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151670543</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1151671051</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>KORKORMALL</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>【国内百貨店】ルラボベルガモット22オードパルファム15ml</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LE LABO</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>19280</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="b">
+        <v>0</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151671051</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J81"/>
+  <autoFilter ref="A1:J96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 15, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$112</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J96"/>
+  <dimension ref="A1:J112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4391,8 +4391,664 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1204368140</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>CosmeticsNo1</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ラディアンソーム100マイクロフルーダイザトナー＋エッセンス</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>21500</v>
+      </c>
+      <c r="G97" t="n">
+        <v>2</v>
+      </c>
+      <c r="H97" t="b">
+        <v>0</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204368140</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1212645182</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>CosmeticsNo1</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>[1+1+1]ボルフィリン 20% アンプルスティック 10ml x 3EA</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G98" t="n">
+        <v>0</v>
+      </c>
+      <c r="H98" t="b">
+        <v>0</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212645182</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1212154060</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>CosmeticsNo1</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>[1+1+1]トラネキサム酸6%クリーム, 30ml x 3EA</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="b">
+        <v>0</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212154060</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1212147421</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>CosmeticsNo1</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>[1+1]トラネキサム酸6%クリーム, 30ml x 2EA</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>1750</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" t="b">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212147421</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1199006617</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Jurian</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>アゼライン酸16BBカーミングセラム, 30ml</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>2578</v>
+      </c>
+      <c r="G101" t="n">
+        <v>1</v>
+      </c>
+      <c r="H101" t="b">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199006617</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1199701690</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Jurian</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>カーミング バランスジェル 100ml / 水分バランス 調節</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>4735</v>
+      </c>
+      <c r="G102" t="n">
+        <v>0</v>
+      </c>
+      <c r="H102" t="b">
+        <v>0</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199701690</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1192507748</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>megadepartment</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>[国内発送]超低分子ヒアルロン酸トナー300ml/オニオンニューペアゲルクリーム50ml/ヒアルロン酸化粧水 ヒアルロン酸トナー/水分 保湿 潤い 乾燥肌 混合肌/韓国コスメ 韓国スキンケア[選択]</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>イズエンツリー</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G103" t="n">
+        <v>3</v>
+      </c>
+      <c r="H103" t="b">
+        <v>0</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192507748</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1202278739</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>megadepartment</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>THE VITA A PDRN レチナールショット タイトニングブースター 20g / PDRN レチナール スポットクリーム / ハリ 弾力ケア 毛穴ケア シワ改善 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>MABUP YEOSHIN</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1680</v>
+      </c>
+      <c r="G104" t="n">
+        <v>1</v>
+      </c>
+      <c r="H104" t="b">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202278739</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1210416288</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>coscoskorea</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>カーミングバランスジェル 100ml</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G105" t="n">
+        <v>0</v>
+      </c>
+      <c r="H105" t="b">
+        <v>0</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210416288</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1210395714</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>coscoskorea</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>クレンジングパウダーウォッシュ 80g</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>4490</v>
+      </c>
+      <c r="G106" t="n">
+        <v>0</v>
+      </c>
+      <c r="H106" t="b">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210395714</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1210367966</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>coscoskorea</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ツーフェイスオイルミスト 50ml</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>5250</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="b">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210367966</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>1064699032</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>hy_international</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>ウォータープルーフプロサンクリーム50g SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>BUSHMAN</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>2599</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="b">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1064699032</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1076432453</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>hy_international</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>ヘアクッション 15g x 2</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>lala chuu</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>3599</v>
+      </c>
+      <c r="G109" t="n">
+        <v>2</v>
+      </c>
+      <c r="H109" t="b">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1076432453</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1194137779</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>プラセン マジックシステム セット 1剤 / 2剤 200ml / 2種 1択</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>ルネセル</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>7058</v>
+      </c>
+      <c r="G110" t="n">
+        <v>1</v>
+      </c>
+      <c r="H110" t="b">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194137779</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1194137521</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>ルティナー マルチバーム 15ml 2個</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>8018</v>
+      </c>
+      <c r="G111" t="n">
+        <v>0</v>
+      </c>
+      <c r="H111" t="b">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194137521</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1172240115</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>COSNRM</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>ダーマジェン イジェンシア 25g 2個 / 50g 2個 / 2種 1択 / 肌の回復と鎮静をサポートする集中保湿クリーム</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Dermagen</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>3956</v>
+      </c>
+      <c r="G112" t="n">
+        <v>6</v>
+      </c>
+      <c r="H112" t="b">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172240115</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J96"/>
+  <autoFilter ref="A1:J112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 18, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J112"/>
+  <dimension ref="A1:J128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5047,8 +5047,664 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1179913892</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>マミケア ビビリップ LED リップ グロウ リップマスク 1個ケースリップバーム 2種乾電池</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Mommy Care</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>7420</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="b">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179913892</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1180095461</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>イーロン アンプル 50ml センシエンド</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>15970</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="b">
+        <v>0</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095461</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1180095290</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>KOREAHUB</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>イーロン ダンギ クレンジングジェル 200ml + 贈呈:マスクパック1枚</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>ILLON</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>6550</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="b">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180095290</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1171638753</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>UKB</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ソウル 1988 セラム: レチナール リポソーム 2% + ブラックジンセン 30ml</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>K-SECRET</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G116" t="n">
+        <v>1</v>
+      </c>
+      <c r="H116" t="b">
+        <v>0</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171638753</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1168676299</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>UKB</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>モイスチャー·レイヤ·サン·プロテクター50ml SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G117" t="n">
+        <v>9</v>
+      </c>
+      <c r="H117" t="b">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168676299</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1187961763</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>[2026] NEW 最低特典カーミング バランスジェル-保湿 / 鎮静 100ml(1+1)</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>10057</v>
+      </c>
+      <c r="G118" t="n">
+        <v>3</v>
+      </c>
+      <c r="H118" t="b">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187961763</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1174936338</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>プリジュビネーション ファーミングバクチオールセラム[童顔弾力セラム] 50ml</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>6902</v>
+      </c>
+      <c r="G119" t="n">
+        <v>0</v>
+      </c>
+      <c r="H119" t="b">
+        <v>0</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174936338</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1208171928</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>[2026BEST] ザマトロジー 2種 セット-光彩 / 弾力(ブースター130ml+セラム45ml)</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>13046</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="b">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208171928</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>1210644303</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>on_j4052</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>【NEW】SW19 ヘアパフュームミスト 75ml 5pm 8am 2種から選べる1種 ヘアミスト ヘアフレグランス 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>SW19</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>5490</v>
+      </c>
+      <c r="G121" t="n">
+        <v>0</v>
+      </c>
+      <c r="H121" t="b">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210644303</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>1210988490</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>[正規品] SET VQM Phytocin VIBANQM LOTION 30ml + フィニッシュローション20ml</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>11780</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="b">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210988490</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>1212008071</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>[正規品] ナチュラル毛穴カバー乳液 韓国正規品</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>オブジェ</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>3070</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="b">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212008071</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>1211131806</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>[公式販売店] ザマトロジー 2種セット[ブースター+セラム]/韓国化粧品</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>11970</v>
+      </c>
+      <c r="G124" t="n">
+        <v>1</v>
+      </c>
+      <c r="H124" t="b">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211131806</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>1211312549</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>[公式販売店] 【1+1】 低刺激ディープクレンジング モイスチャー クレンジングオイル 145ml</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>7790</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="b">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211312549</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>1211131359</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>[公式販売店] ICD 3種 ラジアンソーム100トナー/クリーム/エッセンス</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>29990</v>
+      </c>
+      <c r="G126" t="n">
+        <v>0</v>
+      </c>
+      <c r="H126" t="b">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211131359</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>1177131836</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>koreahubshop</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>ドクターヘディソンピュア100％ビタミンCパウダー50gアンプルトナービタケア</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Dr. Hedison</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>4560</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="b">
+        <v>0</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177131836</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>1189937314</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>koreahubshop</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>アノブ ディープ ダメージ リペア シャンプー 1 + 1 ダブルセット 500ml+500ml</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>4840</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="b">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189937314</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J112"/>
+  <autoFilter ref="A1:J128"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 21, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$128</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J128"/>
+  <dimension ref="A1:J141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5703,8 +5703,541 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1189781351</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>YOUSTUDIO</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>ブライタミン V7トーニング ライトクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>5299</v>
+      </c>
+      <c r="G129" t="n">
+        <v>0</v>
+      </c>
+      <c r="H129" t="b">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189781351</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>1196020481</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>NDY</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>ツーフェイス オイルミスト 50ml 1個 基礎化粧品 保湿 潤い 艶肌 油水分バランス [並行輸入品]</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>4980</v>
+      </c>
+      <c r="G130" t="n">
+        <v>2</v>
+      </c>
+      <c r="H130" t="b">
+        <v>0</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196020481</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>1208338165</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>AnchorBlue</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>[サロン級ホームケア] エクストリーム ダメージ クリニック ヘア アンプル 10ml 9個入り / 傷んだ髪 高濃縮 補修 保湿 ツヤ髪 トリートメント 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>ケラシス</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>3818</v>
+      </c>
+      <c r="G131" t="n">
+        <v>0</v>
+      </c>
+      <c r="H131" t="b">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208338165</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>1209905054</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>ホワイトアプリコット ソリッドパフューム 塗る固体香水 フレグランス 携帯用 30ml</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LUAFEE</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>2499</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="b">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905054</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1209905260</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>オドール オールインワン クリアボディウォッシュ 2個, 460ml</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Nodor</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>7665</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" t="b">
+        <v>0</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905260</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1209905066</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>hiseller</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>ポケモンエディションクリアボディミスト 200ml 企画 (ミニチュア 30ml + イーブイ防水パック)</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>NOT4U</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>3831</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0</v>
+      </c>
+      <c r="H134" t="b">
+        <v>0</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209905066</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>1208411222</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>keto88</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>ブラーフィニッシュサンクッション,リフィル</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>TOCOBO</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>1880</v>
+      </c>
+      <c r="G135" t="n">
+        <v>2</v>
+      </c>
+      <c r="H135" t="b">
+        <v>0</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208411222</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>1173120891</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>vivienpink_SG_jp</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>魔女工場 ピュア クレンジングティッシュ</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G136" t="n">
+        <v>0</v>
+      </c>
+      <c r="H136" t="b">
+        <v>0</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173120891</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>1174362545</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>vivienpink_SG_jp</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>ブライトニング毛穴ジャブティパッド本品40枚+10枚（追加贈呈）</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G137" t="n">
+        <v>3</v>
+      </c>
+      <c r="H137" t="b">
+        <v>0</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174362545</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>1201547339</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>RARI</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>パフュームハンドクリーム [ハローキティ], 50ml</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>ヘトラス</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>2170</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" t="b">
+        <v>0</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201547339</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>1158151170</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>royalshop</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>【NEW】 ドクダミ センテラ レッドスポット クリーム 韓国コスメ 30g</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>2824</v>
+      </c>
+      <c r="G139" t="n">
+        <v>4</v>
+      </c>
+      <c r="H139" t="b">
+        <v>0</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158151170</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>1155003250</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>royalshop</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>つや米 トーンアップ 水分 サンクリーム 日焼け止め 化粧下地 UVカット SPF50+ PA++++ 韓国コスメ [ロイヤルショップ] 100mL</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>シンムルナラ</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>3413</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="b">
+        <v>0</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155003250</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>1157009011</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>royalshop</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>エアライン KF94 黄砂・飛沫対策 3Dマスク 大型サイズ 韓国マスク 100枚セット（25枚×4袋）［ホワイト/ブラック］</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>URBANWIZ</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>2477</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" t="b">
+        <v>0</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157009011</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J128"/>
+  <autoFilter ref="A1:J141"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 24, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$151</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J141"/>
+  <dimension ref="A1:J151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6236,8 +6236,418 @@
         </is>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>1207716735</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>sowoojushop</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>ハニー＆マカダミア ピュアボディローション アカシアモリンガの香り 500ml 韓国ボディケア 保湿ケア しっとり ボディミルク</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>2705</v>
+      </c>
+      <c r="G142" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" t="b">
+        <v>0</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207716735</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>1163853917</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>theonetrade</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>緊急鎮静・敏感肌ケア / 韓国スパ品質の陶器肌クリーム P401 リリーフクリーム 50mL</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Eclat du teint</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>9900</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" t="b">
+        <v>0</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163853917</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>1149797233</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>theonetrade</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>韓国発の人気商品 SW19 ミニ香水お試しセット 3mL X 4本セット</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>SW19</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G144" t="n">
+        <v>2</v>
+      </c>
+      <c r="H144" t="b">
+        <v>0</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149797233</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>1149301635</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>theonetrade</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>韓国で人気のスキンケア5点セットRENEW-AGE スキンケアトナー130mL + 乳液130mL + 美容液30mL + クリーム50mL + アイクリーム20mL ギフトとしても大人気</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>9500</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="b">
+        <v>0</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149301635</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>934718142</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>theonetrade</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>トラブルソープドクダミ石鹸 手作り石鹸100g 1+1/ニキビケア/皮脂コントロール/優しい使い心地/韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LANOA</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>3999</v>
+      </c>
+      <c r="G146" t="n">
+        <v>1</v>
+      </c>
+      <c r="H146" t="b">
+        <v>0</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=934718142</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>1120312659</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>kinakomall</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Glycolic Acid 7% Exfoliating Toner グリコリックアシッド7%エクスポリエイティングトナー(Toning Solution) 100ml, 240ml / グリコリック</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>1789</v>
+      </c>
+      <c r="G147" t="n">
+        <v>8</v>
+      </c>
+      <c r="H147" t="b">
+        <v>0</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1120312659</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>1193462376</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>kinakomall</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>ベータグルカン パワーモイスチャーセラム 50ml</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>iUNIK</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>3408</v>
+      </c>
+      <c r="G148" t="n">
+        <v>2</v>
+      </c>
+      <c r="H148" t="b">
+        <v>0</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193462376</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>1211134600</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>seimyongkorea</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>【NEW】 シェイキングミスト</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>2222</v>
+      </c>
+      <c r="G149" t="n">
+        <v>2</v>
+      </c>
+      <c r="H149" t="b">
+        <v>0</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211134600</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>1197720706</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>K_Beauty_Station</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>【今だけ限定！企画】キャロットカロテンカーミングウォーターパッド, 60枚</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>スキンフード</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>1964</v>
+      </c>
+      <c r="G150" t="n">
+        <v>3</v>
+      </c>
+      <c r="H150" t="b">
+        <v>0</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197720706</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>1212963285</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>K_Beauty_Station</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>ドクダミBHA ジウゲ ピーリングパッド 70枚(60+10枚) 毛穴ケア 角質ケア 皮脂ケア</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>1764</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="b">
+        <v>0</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212963285</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J141"/>
+  <autoFilter ref="A1:J151"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 27, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$168</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:J168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6646,8 +6646,705 @@
         </is>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>1212713877</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Lulupi</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>【フィー】 シェイキングシナジーミスト 50ml 全3種</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>2654</v>
+      </c>
+      <c r="G152" t="n">
+        <v>1</v>
+      </c>
+      <c r="H152" t="b">
+        <v>0</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212713877</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>1213885966</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Lulupi</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>【ソーナチュラル】 オールデイ ブラー ジェリー プライマー フィクサー 5g</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F153" t="n">
+        <v>2432</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" t="b">
+        <v>0</v>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213885966</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>1180144570</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>PDRN トナー250ml1個</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F154" t="n">
+        <v>3230</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" t="b">
+        <v>0</v>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180144570</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>1202055978</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>UVクリーム SPF50+ PA ++++ 敏感肌向けトーンアップ韓国コスメの人気日焼け止め</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F155" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" t="b">
+        <v>0</v>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202055978</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>1174315936</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>1. マデカラボ マスク 10枚×2箱（リンクル リバイタライズ）</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F156" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G156" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" t="b">
+        <v>0</v>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174315936</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>1183743968</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>zz6o6</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>パーフェクト9 インテンシブ スキンケアセット 化粧水 乳液 クリーム セット スキンケア 保湿 セット 保湿</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F157" t="n">
+        <v>5253</v>
+      </c>
+      <c r="G157" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" t="b">
+        <v>0</v>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183743968</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>1177458353</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>zz6o6</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>コジサン ソープ 65g×3個 フィリピン製 ナチュラル オレンジ石鹸 ギフトにもおすすめ</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>こじえさん</t>
+        </is>
+      </c>
+      <c r="F158" t="n">
+        <v>2232</v>
+      </c>
+      <c r="G158" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" t="b">
+        <v>0</v>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177458353</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>1103721247</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>COREDREAM</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Inner perfume 5ml 14種 / Yゾーンケア /生臭さ除去 / 下着香水</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>フォエリー</t>
+        </is>
+      </c>
+      <c r="F159" t="n">
+        <v>2190</v>
+      </c>
+      <c r="G159" t="n">
+        <v>3</v>
+      </c>
+      <c r="H159" t="b">
+        <v>0</v>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1103721247</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>1191723236</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>ホワイトティ ジンジャーリリー ボディクリーム 400ml</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>エリザベスアーデン</t>
+        </is>
+      </c>
+      <c r="F160" t="n">
+        <v>3344</v>
+      </c>
+      <c r="G160" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" t="b">
+        <v>0</v>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191723236</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>1203745241</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>スキンコンディショナーエッセンシャル 330ml</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>アルビオン</t>
+        </is>
+      </c>
+      <c r="F161" t="n">
+        <v>10106</v>
+      </c>
+      <c r="G161" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" t="b">
+        <v>0</v>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203745241</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>1154890233</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>ロム イデアル インテンス オーデパルファン 100ml</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>ゲラン</t>
+        </is>
+      </c>
+      <c r="F162" t="n">
+        <v>20617</v>
+      </c>
+      <c r="G162" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" t="b">
+        <v>0</v>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154890233</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>1123998991</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>イリシットオーデパルファム 100ml</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>ジミーチュウ</t>
+        </is>
+      </c>
+      <c r="F163" t="n">
+        <v>10654</v>
+      </c>
+      <c r="G163" t="n">
+        <v>0</v>
+      </c>
+      <c r="H163" t="b">
+        <v>0</v>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123998991</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>1163881732</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>ロレアル セリエ ブロンディファイアー マスク 500ml</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F164" t="n">
+        <v>5374</v>
+      </c>
+      <c r="G164" t="n">
+        <v>0</v>
+      </c>
+      <c r="H164" t="b">
+        <v>0</v>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163881732</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>1123944887</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>グリーンティー ボディローション 500ml</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>エリザベスアーデン</t>
+        </is>
+      </c>
+      <c r="F165" t="n">
+        <v>1679</v>
+      </c>
+      <c r="G165" t="n">
+        <v>7</v>
+      </c>
+      <c r="H165" t="b">
+        <v>0</v>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123944887</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>1204380898</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>ニューバーム ソフトムスク 40g</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>RETOUCH</t>
+        </is>
+      </c>
+      <c r="F166" t="n">
+        <v>2809</v>
+      </c>
+      <c r="G166" t="n">
+        <v>0</v>
+      </c>
+      <c r="H166" t="b">
+        <v>0</v>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204380898</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>1189355281</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>beautyofkorea</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>ドクダミ77％ 化粧水 250ml</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F167" t="n">
+        <v>1761</v>
+      </c>
+      <c r="G167" t="n">
+        <v>0</v>
+      </c>
+      <c r="H167" t="b">
+        <v>0</v>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189355281</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>1131933510</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>K-Aesthetique</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>セルマン ビタミンC セラム 30ml Vitamin C Serum エステサロン専用 韓国化粧品</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>SERMENT</t>
+        </is>
+      </c>
+      <c r="F168" t="n">
+        <v>8300</v>
+      </c>
+      <c r="G168" t="n">
+        <v>5</v>
+      </c>
+      <c r="H168" t="b">
+        <v>0</v>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1131933510</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J151"/>
+  <autoFilter ref="A1:J168"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 30, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$168</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$186</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J168"/>
+  <dimension ref="A1:J186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7343,8 +7343,746 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>1197392833</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>KOKOkr</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>PDRNデイリーマスク 30枚</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F169" t="n">
+        <v>1599</v>
+      </c>
+      <c r="G169" t="n">
+        <v>7</v>
+      </c>
+      <c r="H169" t="b">
+        <v>0</v>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197392833</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>1196376380</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>KOKOkr</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>マダガスカルセンテラヒアル-シカシルキーフィットサンスティック 20g SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F170" t="n">
+        <v>1599</v>
+      </c>
+      <c r="G170" t="n">
+        <v>8</v>
+      </c>
+      <c r="H170" t="b">
+        <v>0</v>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196376380</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>1172550313</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>KOKOkr</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>PDRNピンクペプチドアンプルリフィル50ml / 1個</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F171" t="n">
+        <v>1649</v>
+      </c>
+      <c r="G171" t="n">
+        <v>4</v>
+      </c>
+      <c r="H171" t="b">
+        <v>0</v>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172550313</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>1157524219</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>バイオEXセルペプチド3種セット1個 水分・保湿・栄養・肌のハリ・シワケア</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>トニーモリー</t>
+        </is>
+      </c>
+      <c r="F172" t="n">
+        <v>5979</v>
+      </c>
+      <c r="G172" t="n">
+        <v>0</v>
+      </c>
+      <c r="H172" t="b">
+        <v>0</v>
+      </c>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157524219</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>1149796005</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>センテラ トーニングトナー 鎮静 シカ 化粧水 210ml</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F173" t="n">
+        <v>1974</v>
+      </c>
+      <c r="G173" t="n">
+        <v>0</v>
+      </c>
+      <c r="H173" t="b">
+        <v>0</v>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1149796005</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>1172781112</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>[3点セット/企画構成/復活草マスクパック1枚贈呈]復活草 パハトナー200ml+復活草 ビフィダ セラム ファーミング ドロップ 50ml+復活草 クリーム ニュートリション チューブ 75ml</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F174" t="n">
+        <v>5819</v>
+      </c>
+      <c r="G174" t="n">
+        <v>0</v>
+      </c>
+      <c r="H174" t="b">
+        <v>0</v>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172781112</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>1155298751</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>【リニューアル】ゼロ毛穴 ワンデーセラム 30ml 1本 毛穴ケア 肌のキメ</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F175" t="n">
+        <v>2348</v>
+      </c>
+      <c r="G175" t="n">
+        <v>0</v>
+      </c>
+      <c r="H175" t="b">
+        <v>0</v>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1155298751</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>1151012307</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>KLand</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>ドクダミポアコントロールクレンジングオイル 200ml</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F176" t="n">
+        <v>2691</v>
+      </c>
+      <c r="G176" t="n">
+        <v>1</v>
+      </c>
+      <c r="H176" t="b">
+        <v>0</v>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151012307</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>1163428866</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>kspecial</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>キュスカゲル 10g ビタミンE 配合 ステロイド無添加 ケロイド 肥厚性瘢痕 ニキビ跡医療用シリコンゲル 手術・火傷・外傷 傷跡管理</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F177" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G177" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" t="b">
+        <v>0</v>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163428866</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>1162958747</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>topkorea</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>リアルマットメイクアップセッティングフィックスミスト75ml フィクサー メイクキープミスト メイクキープスプレー /韓国コスメ 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F178" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G178" t="n">
+        <v>6</v>
+      </c>
+      <c r="H178" t="b">
+        <v>0</v>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162958747</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>1083980822</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>topkorea</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>セラミドアト6.0 トップトゥトー全身ウォッシュ 1000ml</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>イリユン</t>
+        </is>
+      </c>
+      <c r="F179" t="n">
+        <v>2732</v>
+      </c>
+      <c r="G179" t="n">
+        <v>0</v>
+      </c>
+      <c r="H179" t="b">
+        <v>0</v>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1083980822</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>1167024145</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>topkorea</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>ホワイトトリュフファーストスプレーセラム 100ml /150ml 保湿/栄養/弾力/ハリ/光彩/ツヤ/</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F180" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G180" t="n">
+        <v>1</v>
+      </c>
+      <c r="H180" t="b">
+        <v>0</v>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1167024145</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>1162947006</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>topkorea</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>ガラクナイアシン3.0エッセンス, 60ml, /韓国コスメ 韓国スキンケア</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>manyo</t>
+        </is>
+      </c>
+      <c r="F181" t="n">
+        <v>1590</v>
+      </c>
+      <c r="G181" t="n">
+        <v>4</v>
+      </c>
+      <c r="H181" t="b">
+        <v>0</v>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162947006</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>1209235398</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿クリーム 50ml 韓国コスメ 韓国ブランド 公式ショップ 韓国スキンケア スキンケア 化粧品 敏感肌 乾燥肌 水分ケア うるおい 韓国アンプル ギフト PDRN CICA</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F182" t="n">
+        <v>2664</v>
+      </c>
+      <c r="G182" t="n">
+        <v>0</v>
+      </c>
+      <c r="H182" t="b">
+        <v>0</v>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209235398</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>1209222941</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿トナー 150ml 韓国スキンケア 韓国コスメ スキンケア PDRN CICA ヒアルロン酸 水分ケア　乾燥肌 ローション 化粧水 整肌成分 毎日のケア 弱酸性 韓国商品 高保湿</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>2472</v>
+      </c>
+      <c r="G183" t="n">
+        <v>0</v>
+      </c>
+      <c r="H183" t="b">
+        <v>0</v>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209222941</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>1210318709</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿アンプル 30ml 2個セット 1+1 美容液 セラム 韓国コスメ 韓国スキンケア 化粧品 スキンケア PDRN パインショットエクソソーム CICA うるおい 水分 アンプル</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F184" t="n">
+        <v>3336</v>
+      </c>
+      <c r="G184" t="n">
+        <v>0</v>
+      </c>
+      <c r="H184" t="b">
+        <v>0</v>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210318709</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>1209368965</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>エクソソーム保湿パッククレンザー 150ml 洗顔 メイク落とし 乾燥肌 敏感肌 弱酸性 韓国スキンケア 韓国コスメ クレンジング 保湿 泡立ち 2WAY パック 韓国化粧品 韓国 韓国好き</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Oningvibe</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>2454</v>
+      </c>
+      <c r="G185" t="n">
+        <v>0</v>
+      </c>
+      <c r="H185" t="b">
+        <v>0</v>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209368965</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>1190410398</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>lebelage</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>【公式】【1つ選択】トゥルーリートナーパッドシリーズ5種（各60枚入り）／拭き取りパッド／部分パック／肌悩み別トナーパッド／グルタチオン／パンテノール／センテラ／レチノール／時短ケア</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>ルベラジュ</t>
+        </is>
+      </c>
+      <c r="F186" t="n">
+        <v>1710</v>
+      </c>
+      <c r="G186" t="n">
+        <v>0</v>
+      </c>
+      <c r="H186" t="b">
+        <v>0</v>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190410398</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J168"/>
+  <autoFilter ref="A1:J186"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 33, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$186</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$190</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J186"/>
+  <dimension ref="A1:J190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8081,8 +8081,172 @@
         </is>
       </c>
     </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>1168425085</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>lannor</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>ザマデカクリーム (シーズン6), 50ml, 3個 (ボックス無)</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>2752</v>
+      </c>
+      <c r="G187" t="n">
+        <v>1</v>
+      </c>
+      <c r="H187" t="b">
+        <v>0</v>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168425085</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>1151142091</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>vacian</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>【公式】ゴールドシル ペプチド コラーゲン シワ リフティング アンプル 30mlハリ肌・エイジングケア・韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>VACIAN</t>
+        </is>
+      </c>
+      <c r="F188" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G188" t="n">
+        <v>0</v>
+      </c>
+      <c r="H188" t="b">
+        <v>0</v>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1151142091</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>1140049631</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>vacian</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>【公式】 目元リフティング スピキュール ペプチド アイクリーム 15ml たるみ・シワ・エイジングケア・韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>VACIAN</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G189" t="n">
+        <v>2</v>
+      </c>
+      <c r="H189" t="b">
+        <v>0</v>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1140049631</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>1183673001</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>t-garden</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>【OUTLET】 シースルーグロス 【COOL】【WARM】シャンプー / トリートメント ボトル</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>RASICA</t>
+        </is>
+      </c>
+      <c r="F190" t="n">
+        <v>1584</v>
+      </c>
+      <c r="G190" t="n">
+        <v>0</v>
+      </c>
+      <c r="H190" t="b">
+        <v>0</v>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183673001</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J186"/>
+  <autoFilter ref="A1:J190"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 1, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$307</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$320</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J307"/>
+  <dimension ref="A1:J320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13042,8 +13042,541 @@
         </is>
       </c>
     </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>1094120054</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>【日本公式代理店】韓国 アイクリーム レチノコラーゲン低分子300集中クリーム レチノール レチナール 目元たるみ 30代 40代 50代 低分子フィッシュコラーゲン しわ 目尻 ほうれい 人気</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>CKD_GUARANTEED</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" t="b">
+        <v>0</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094120054</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>1145826907</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>【公式】ウォーターフィット サンセラム 日焼け止め 国内発送 シカ センテラ 韓国コスメ 水分 保湿 鎮静 低刺激 UVカット 化粧下地 紫外線</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>2530</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="b">
+        <v>0</v>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145826907</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>1175765151</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>【公式】Vita 3 ACE Aurora Toner 化粧水 保湿 ビタミン インナードライ スキンケア 韓国コスメ 水光肌 トーンアップ ニキビ跡ケア 国内発送</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>オーズナリー</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G310" t="n">
+        <v>3</v>
+      </c>
+      <c r="H310" t="b">
+        <v>0</v>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175765151</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>1175759418</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>【公式】 【LDK受賞】 Vita 3 BBC Pudding Cream ビタミン 跡ケア 保湿 高密着 スキンケア ナイトケア スリーピングパック トーンアップ</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>オーズナリー</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0</v>
+      </c>
+      <c r="H311" t="b">
+        <v>0</v>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175759418</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>1174265093</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>【公式】 プロバイオシカ インテンシブアンプル アンプル 50ml 美容液 鎮静 保湿 バリア ケア スキンケア センテラ ツボクサ　国内発送</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G312" t="n">
+        <v>4</v>
+      </c>
+      <c r="H312" t="b">
+        <v>0</v>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174265093</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>1100332949</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>balifesta</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>サンスクリーン Daily Refreshing Serum SPF50+ PA++++ 170ml 海外直送品</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>ヴァセリン</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>3690</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" t="b">
+        <v>0</v>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1100332949</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>1208319671</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>balifesta</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Mugwort　Acne Clay Stick　40g</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>SKINTIFIC</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>4990</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0</v>
+      </c>
+      <c r="H314" t="b">
+        <v>0</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208319671</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>1208182736</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>balifesta</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>PDRN シリーズ　Radiance Bright Serum Spray　100ml</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>SKINTIFIC</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>5590</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0</v>
+      </c>
+      <c r="H315" t="b">
+        <v>0</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208182736</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>1191796909</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>lamelin</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>【キメ・しっとり・なめらか】ラメリン ミラクルNMNプラスPDRN バイオトックス クリーム 50ml シワ毛穴ケア(NMN/PDRN)</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LAMELIN</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>3070</v>
+      </c>
+      <c r="G316" t="n">
+        <v>15</v>
+      </c>
+      <c r="H316" t="b">
+        <v>0</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191796909</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>1203108437</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>reveam</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>リブエム ウォーターフィット 8重保湿トナーパッド 詰め替え 角質ケア 保湿 30枚</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Reve:am</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>1630</v>
+      </c>
+      <c r="G317" t="n">
+        <v>0</v>
+      </c>
+      <c r="H317" t="b">
+        <v>0</v>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203108437</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>1206155481</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>beiskin</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>【ハリ密着】ローズウォーター コラーゲン マスク 500Da 超低分子 10枚入</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>beiskin</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>4980</v>
+      </c>
+      <c r="G318" t="n">
+        <v>3</v>
+      </c>
+      <c r="H318" t="b">
+        <v>0</v>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206155481</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>1203211333</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>BRMUD_Official</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>【公式】 リカバリーマッドスクラブデイリーウォッシュ 500ml／ボディソープ／ボディウォッシュ／天然泥スクラブ／背中ニキビ／角質ケア／なめらかシルク肌／お風呂</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>BRMUD</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G319" t="n">
+        <v>13</v>
+      </c>
+      <c r="H319" t="b">
+        <v>0</v>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203211333</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>1145867764</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>BRMUD_Official</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>【公式】リリーフマッドマスク200ML／洗い流す泥パック／クレイパック／毛穴・角質ケア／黒ずみ／ピーリング／ニキビケア／皮脂撲滅／ゆでたまご肌</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>BRMUD</t>
+        </is>
+      </c>
+      <c r="F320" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G320" t="n">
+        <v>14</v>
+      </c>
+      <c r="H320" t="b">
+        <v>0</v>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145867764</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J307"/>
+  <autoFilter ref="A1:J320"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 2, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$320</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$334</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J320"/>
+  <dimension ref="A1:J334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13575,8 +13575,582 @@
         </is>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>1104732964</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>idplacosmeticsofficial</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>【正規品】　id フェイスフィットSLバンドV2　【10枚セット】　【下あごケア用】　イヤーリングタイプ　マイナスバンド　接着剤無し　100％ハイドロジェル　韓国最大の美容整形外科開発</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>id PLACOSMETICS</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>5500</v>
+      </c>
+      <c r="G321" t="n">
+        <v>1</v>
+      </c>
+      <c r="H321" t="b">
+        <v>0</v>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1104732964</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>1184935545</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>tomocos</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>ブダペスト ボディーローション 300ml</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>raconteur</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G322" t="n">
+        <v>0</v>
+      </c>
+      <c r="H322" t="b">
+        <v>0</v>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1184935545</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>1184934871</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>tomocos</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>バンフ ボディオイル 150ml</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>raconteur</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0</v>
+      </c>
+      <c r="H323" t="b">
+        <v>0</v>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1184934871</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>1152365470</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>puremax</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>ハイエンド SPF50 スパ 日焼け止め 1個</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LBB</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>4330</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0</v>
+      </c>
+      <c r="H324" t="b">
+        <v>0</v>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152365470</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>1152911535</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>puremax</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>ー グリーントマト フォア リフティング アンプル 75ml 1個</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>Sung Boon Editor</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G325" t="n">
+        <v>2</v>
+      </c>
+      <c r="H325" t="b">
+        <v>0</v>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1152911535</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>1209815486</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>uiq-japan</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>【新発売】バイオームレメディポアリセットクーリングPDRNハイドロゲルマスク5枚セット #肌クールダウン #毛穴ケア #化粧ノリUP</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>UIQ</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G326" t="n">
+        <v>7</v>
+      </c>
+      <c r="H326" t="b">
+        <v>0</v>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209815486</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>1170053960</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>mayo</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>プロテイン ダメージケア バイオレット ミュゲの香り / アイリッシュ/イランイラン 3つの香り シャンプー500ml + トリートメント250ml</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Kundal</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>3090</v>
+      </c>
+      <c r="G327" t="n">
+        <v>7</v>
+      </c>
+      <c r="H327" t="b">
+        <v>0</v>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170053960</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>1211377983</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>GODONSHOP</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>KIEHL’S キールズ レアアース マスク 125mL フェイスマスク</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>キールズ</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>4390</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0</v>
+      </c>
+      <c r="H328" t="b">
+        <v>0</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211377983</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>1208526902</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>GODONSHOP</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>KIEHL’S キールズ クリーム UFC クリーム 125mL 大容量 保湿 クリーム</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>キールズ</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>6190</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0</v>
+      </c>
+      <c r="H329" t="b">
+        <v>0</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208526902</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>1211377673</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>GODONSHOP</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>KIEHL’S キールズ DSクリアリーブライト エッセンス 美容液 100ml 115ml</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>キールズ</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>16990</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0</v>
+      </c>
+      <c r="H330" t="b">
+        <v>0</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211377673</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>984679415</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>beauty_sky</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>round lab 韓国sns話題_白樺水分トナー300ml_韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>2850</v>
+      </c>
+      <c r="G331" t="n">
+        <v>6</v>
+      </c>
+      <c r="H331" t="b">
+        <v>0</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=984679415</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>984679124</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>beauty_sky</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>round lab 韓国sns話題_シラカバ水分クリーム80ml_韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>3249</v>
+      </c>
+      <c r="G332" t="n">
+        <v>10</v>
+      </c>
+      <c r="H332" t="b">
+        <v>0</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=984679124</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>1208272693</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>furriky</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>[GIFT SET] ヘアミスト グロー Belle ＆ ピンクファーリー ポーチキーリング</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>Furriky</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>5617</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="b">
+        <v>0</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208272693</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>1211534870</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>seoullife</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>ジャムパッククレンザー 120ml</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>earfit</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>2750</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
+      <c r="H334" t="b">
+        <v>0</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211534870</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J320"/>
+  <autoFilter ref="A1:J334"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 4, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$343</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$344</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J343"/>
+  <dimension ref="A1:J344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14518,8 +14518,49 @@
         </is>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>1121008564</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>smartselect</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>フォーマント シグネチャー コットンスプレー コットンハグ 200ml</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>FORMENT</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>4780</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0</v>
+      </c>
+      <c r="H344" t="b">
+        <v>0</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1121008564</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J343"/>
+  <autoFilter ref="A1:J344"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 7, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$347</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$350</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J347"/>
+  <dimension ref="A1:J350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14682,8 +14682,131 @@
         </is>
       </c>
     </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>1209053534</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>【公式/新発売】カーミング トラベルキット+(*カート番号ごとに一つ)シャシェ2種</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>2880</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0</v>
+      </c>
+      <c r="H348" t="b">
+        <v>0</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209053534</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>1205876934</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>【公式】バランスリカバリーマスク1枚+(*カート番号ごとに一つ)シャシェ2種</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>378</v>
+      </c>
+      <c r="G349" t="n">
+        <v>7</v>
+      </c>
+      <c r="H349" t="b">
+        <v>0</v>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205876934</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>1200670476</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>[公式]エアリー デュ サン セラム+(*カート番号ごとに一つ)シャシェ2種</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Lowlize</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>2736</v>
+      </c>
+      <c r="G350" t="n">
+        <v>5</v>
+      </c>
+      <c r="H350" t="b">
+        <v>0</v>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200670476</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J347"/>
+  <autoFilter ref="A1:J350"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 10, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$350</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$353</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J350"/>
+  <dimension ref="A1:J353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14805,8 +14805,131 @@
         </is>
       </c>
     </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>1099343162</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>sopo</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>【夏のヘアケア福袋】by Yarden バイヤーデン ダメージケア シャンプー2個&amp;amp;トリートメント2個&amp;amp;スカルプリリーフセラムセット</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>by yarden</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>4284</v>
+      </c>
+      <c r="G351" t="n">
+        <v>3</v>
+      </c>
+      <c r="H351" t="b">
+        <v>0</v>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1099343162</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>1200195801</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>sopo</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>【ダメージケア】by Yarden バイヤーデン ダメージケア ダメージヘア 補修 シャンプー&amp;amp;トリートメント</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>by yarden</t>
+        </is>
+      </c>
+      <c r="F352" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G352" t="n">
+        <v>9</v>
+      </c>
+      <c r="H352" t="b">
+        <v>0</v>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200195801</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>1201956239</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>sopo</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>【ヘアセラム】by Yarden バイヤーデン スカルプ リリーフ セラム</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>by yarden</t>
+        </is>
+      </c>
+      <c r="F353" t="n">
+        <v>2400</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0</v>
+      </c>
+      <c r="H353" t="b">
+        <v>0</v>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201956239</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J350"/>
+  <autoFilter ref="A1:J353"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 11)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$353</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$358</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J353"/>
+  <dimension ref="A1:J358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14928,8 +14928,213 @@
         </is>
       </c>
     </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>1203847132</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>hairtheory-lab</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>【公式】【べスコス多数受賞】ヘアセオリーラボ フューチャー バイタル エッセンス / 50mL / 正規品 / 頭皮美容液 スカルプケア 頭皮ケア ボリュームケア ハリ コシ エイジングケア 美髪</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Hair Theory Lab</t>
+        </is>
+      </c>
+      <c r="F354" t="n">
+        <v>7920</v>
+      </c>
+      <c r="G354" t="n">
+        <v>1</v>
+      </c>
+      <c r="H354" t="b">
+        <v>0</v>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203847132</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>1191440176</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>hairtheory-lab</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>【公式】ヘアセオリーラボ セラムイン オイル アウトバストリートメント / 95ml / Hair Theory Lab 正規品 / 洗い流さないトリートメント アウトバスヘアケア ダメージケア</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Hair Theory Lab</t>
+        </is>
+      </c>
+      <c r="F355" t="n">
+        <v>5940</v>
+      </c>
+      <c r="G355" t="n">
+        <v>16</v>
+      </c>
+      <c r="H355" t="b">
+        <v>0</v>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191440176</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>1156253951</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>hairtheory-lab</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>【公式】ヘアセオリーラボ セラムイン トリートメント / 300ml / 正規品 / うねり くせ毛 パサつき 乾燥 ダメージケア ハリ コシ ツヤ 輝き うるおい まとまり 美容液</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Hair Theory Lab</t>
+        </is>
+      </c>
+      <c r="F356" t="n">
+        <v>5500</v>
+      </c>
+      <c r="G356" t="n">
+        <v>3</v>
+      </c>
+      <c r="H356" t="b">
+        <v>0</v>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156253951</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>1156248781</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>hairtheory-lab</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>【公式】ヘアセオリーラボ セラムイン シャンプー / 300ml / 正規品 / うねり くせ毛 パサつき 乾燥 ダメージケア ハリ コシ ツヤ 輝き うるおい まとまり 美容液</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Hair Theory Lab</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>5060</v>
+      </c>
+      <c r="G357" t="n">
+        <v>5</v>
+      </c>
+      <c r="H357" t="b">
+        <v>0</v>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156248781</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>1139722127</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>beans</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>エッセンスＶ シャンプー 1000ml</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>イオニート</t>
+        </is>
+      </c>
+      <c r="F358" t="n">
+        <v>8800</v>
+      </c>
+      <c r="G358" t="n">
+        <v>12</v>
+      </c>
+      <c r="H358" t="b">
+        <v>0</v>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1139722127</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J353"/>
+  <autoFilter ref="A1:J358"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 8, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$363</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$366</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J363"/>
+  <dimension ref="A1:J366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15338,8 +15338,131 @@
         </is>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>1190007692</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>bespoir</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>peau de Reve（ポードレーヴ） トリプルVCローション 100mL＋MOUクリーム 50g 日本製 セラミド ビタミンC 誘導体 アラントイン ナイアシンアミド うるおい 化粧水 クリーム</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>peau de Reve</t>
+        </is>
+      </c>
+      <c r="F364" t="n">
+        <v>9450</v>
+      </c>
+      <c r="G364" t="n">
+        <v>1</v>
+      </c>
+      <c r="H364" t="b">
+        <v>0</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190007692</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>1188455744</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>bespoir</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>peau de Reve（ポードレーヴ） MOUクリーム 50g 日本製 クリーム セラミド ガラクトミセス グリチルリチン酸 トコフェリルリン酸 うるおい 顔 フェイシャル スキンケア 保湿 乾燥</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>peau de Reve</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>2970</v>
+      </c>
+      <c r="G365" t="n">
+        <v>2</v>
+      </c>
+      <c r="H365" t="b">
+        <v>0</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188455744</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>1188455621</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>bespoir</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>peau de Reve（ポードレーヴ）トリプルVCローション 100mL 日本製 化粧水 ビタミンC 誘導体 ナイアシンアミド アラントイン うるおい</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>peau de Reve</t>
+        </is>
+      </c>
+      <c r="F366" t="n">
+        <v>6980</v>
+      </c>
+      <c r="G366" t="n">
+        <v>1</v>
+      </c>
+      <c r="H366" t="b">
+        <v>0</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188455621</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J363"/>
+  <autoFilter ref="A1:J366"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 4)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$376</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$377</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J376"/>
+  <dimension ref="A1:J377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15871,8 +15871,49 @@
         </is>
       </c>
     </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>1198755469</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>kiwiglow</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>ビーガンジェジュ 蓮マイルド角質ケアトナーパッド</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>KIWIGLOW</t>
+        </is>
+      </c>
+      <c r="F377" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G377" t="n">
+        <v>1</v>
+      </c>
+      <c r="H377" t="b">
+        <v>0</v>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198755469</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J376"/>
+  <autoFilter ref="A1:J377"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 5, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$377</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$378</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J377"/>
+  <dimension ref="A1:J378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -15912,8 +15912,49 @@
         </is>
       </c>
     </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>1044468382</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>raftelcosmetic</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>【公式】インテンシブ PM 10 セラム 30ml シワ 夜用 美容液 高濃縮 弾力 抗酸化 ナイアシンアミド スクアラン ヒアルロン酸</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>RAFTEL</t>
+        </is>
+      </c>
+      <c r="F378" t="n">
+        <v>7300</v>
+      </c>
+      <c r="G378" t="n">
+        <v>15</v>
+      </c>
+      <c r="H378" t="b">
+        <v>0</v>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1044468382</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J377"/>
+  <autoFilter ref="A1:J378"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 10 own-file progress (반복 8)
</commit_message>
<xml_diff>
--- a/output/discovery_result_10.xlsx
+++ b/output/discovery_result_10.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$411</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$412</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J411"/>
+  <dimension ref="A1:J412"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17306,8 +17306,49 @@
         </is>
       </c>
     </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>1203828339</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>STAR-ONLINE</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>【美容皮膚科医 監修】デリケートゾーンケア オイル 120ml フェムケア ボディオイル 保湿 膣 乾燥 黒ずみ くすみ 臭い マッサージ 更年期 閉経 かゆみ 産後 会陰 陰部 VIO バスト</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>CHILL CHER</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G412" t="n">
+        <v>6</v>
+      </c>
+      <c r="H412" t="b">
+        <v>0</v>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203828339</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J411"/>
+  <autoFilter ref="A1:J412"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>